<commit_message>
Add reaction GIFs and refactor locale handling
Add a large reaction GIF dataset (assets/reaction_gifs.json and assets/reaction_gifs.py) and simplify/refactor locale-based UI logic across multiple components. Replace repetitive English locale checks with a single not-in ("fr", "de") condition, localize modal labels/embeds, and improve the BotReport flow by normalizing translation-error reports and adding localized input fields. Update constructors and callbacks (Confirmation now receives ctx, ReportModal accepts report title and normalizes type, ModuleMenu signature changed), adjust emoji lookup in Country_Badge_Buttons, and fix a few iteration issues (zip(..., strict=False)). These changes simplify locale branching, improve translation reporting, and add reaction assets; note the changed APIs for Confirmation, ReportModal and ModuleMenu may require callers to be updated.
</commit_message>
<xml_diff>
--- a/commands.xlsx
+++ b/commands.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,31 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date and Time</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>User ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Command Used</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Command Usage</t>
         </is>
@@ -466,19 +454,119 @@
           <t>stacer_varien</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>profile_name</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'profile_name', 'id': '1368684777456144445'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:24:55.766907</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>help_group_name ask</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'options': [{'type': 1, 'options': [{'value': 'how do i use the 8ball command?', 'type': 3, 'name': 'question'}], 'name': 'ask'}], 'name': 'help_group_name', 'id': '1382822284288458882'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:25:13.715069</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>hug_name</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'hug_name', 'id': '1387741616894120026'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:25:37.275103</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>spin_name</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'options': [{'value': 30, 'type': 4, 'name': 'bet_parm_name'}], 'name': 'spin_name', 'id': '1486804616971816970'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:26:19.820277</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>597829930964877369</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>profile_name</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>{'type': 1, 'name': 'profile_name', 'id': '1368684777456144445'}</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>stats</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'stats', 'id': '1368684777456144444'}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor locale handling and improve currency formatting
Replace ctx.locale.value with get_command_locale() function across all cogs for consistent locale detection. Add ServerSettings.format_currency_for() helper to display server-specific currency formatting instead of hardcoded QP references. Implement case ID tracking for all moderation actions (ban, kick, warn, timeout, etc.). Add owner-only currency management commands (qp check/add/remove/set). Update command translations to reference generic 'currency' instead of 'QP'.

This branch is not yet tested
</commit_message>
<xml_diff>
--- a/commands.xlsx
+++ b/commands.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,19 +554,94 @@
           <t>stacer_varien</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>stats</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'stats', 'id': '1368684777456144444'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:37:50.426477</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>spin_name</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'options': [{'value': 30, 'type': 4, 'name': 'bet_parm_name'}], 'name': 'spin_name', 'id': '1486804616971816970'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:38:17.180184</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5.978299309648773e+17</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>hentai</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'hentai', 'id': '1395511830830645293'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:46:15.983789</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>stacer_varien</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>597829930964877369</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>stats</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>{'type': 1, 'name': 'stats', 'id': '1368684777456144444'}</t>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>profile_name</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{'type': 1, 'name': 'profile_name', 'id': '1368684777456144445'}</t>
         </is>
       </c>
     </row>

</xml_diff>